<commit_message>
Update CP learning record after S0-A final FAIL
</commit_message>
<xml_diff>
--- a/records/CP_Learning_Record.xlsx
+++ b/records/CP_Learning_Record.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="R6c939c68a10846e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="R864413c67c8c4c28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="R1c4bc4eb7c2f4168"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="Re2dc3815f65d4c5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="R85a91cf5845541bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="Rf3945651fec74c83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="R5e0dd23ce331468e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="Rcb24622494c64e6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="Re767854e900141e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="R64d610c9006a4d3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="Rd4ac0ac7f8a94731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="R2e4b3d4a5fd642d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="R6fe9475e86c04a26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="R2328eb3985e942e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="Rb69c87f518434876"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="Ra1d3b1592fbb4f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="Rc400ed334d5947b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="Rdd6433c599424e83"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -695,6 +695,92 @@
         <x:v>Clean independent retest. Submitted program compiles and is correct on the sample, boundary-oriented tests, and randomized differential checks. Required helper function is defined and called. O(N) time and O(1) extra-space explanations are correct. No edge case was explicitly listed, but the implementation handles key categories including x&lt;0, x=0, positive even/odd values, N=1, and input bounds; omission of an explicit self-check is retained as a process note rather than a correctness failure. Proceed to Part F final assessment.</x:v>
       </x:c>
     </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>S0-A — C++ Basic Execution</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Final Assessment — Attempt 1</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Longest contiguous nonzero sign-alternating segment</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>Reference execution + exhaustive small-case verification + randomized differential verification</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>R1</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>I2</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>Comparative / Provisional</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>CP_Calibration_Anchor_Registry_v1.1</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>Basic execution: input + conditional branching + loop + helper function + scalar state tracking</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>Incomplete</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="N4"/>
+      <x:c r="O4" t="n">
+        <x:v>28.716666666666665</x:v>
+      </x:c>
+      <x:c r="P4"/>
+      <x:c r="Q4"/>
+      <x:c r="R4"/>
+      <x:c r="S4"/>
+      <x:c r="T4"/>
+      <x:c r="U4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V4" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="W4" t="str">
+        <x:v>FAIL</x:v>
+      </x:c>
+      <x:c r="X4" t="str">
+        <x:v>Correctness</x:v>
+      </x:c>
+      <x:c r="Y4" t="str">
+        <x:v>Important zero-boundary handling failure; first zero counted as length 1; zero/nonzero transition unconditionally resets current length to 0; no edge-case self-check</x:v>
+      </x:c>
+      <x:c r="Z4" t="str">
+        <x:v>L3</x:v>
+      </x:c>
+      <x:c r="AA4" t="str">
+        <x:v>Provisional</x:v>
+      </x:c>
+      <x:c r="AB4" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="AC4" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="AD4" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="AE4" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AF4" t="str">
+        <x:v>Core O(N)/O(1) state-tracking idea is viable and sample/nonzero alternating cases work, but important zero cases fail. Counterexamples: N=1,[0] returns 1 instead of 0; [0,5,-3] returns 1 instead of 2. The duplicated unconditional `sum1 = 0;` inside the zero-product branch erases a valid new length-1 segment when previous value is zero and current value is nonzero. First-element logic also counts zero as a valid segment. First formal final-assessment FAIL; per v5.4 §39.1, convert this problem to learning mode, remediate, then reassess with a new equivalent problem.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -784,7 +870,7 @@
         <x:v>Immediate</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
-        <x:v>Sufficient for Provisional</x:v>
+        <x:v>Incomplete</x:v>
       </x:c>
       <x:c r="H2" s="18" t="str">
         <x:v>None</x:v>
@@ -793,19 +879,19 @@
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="J2" s="18" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="K2" s="18" t="str">
         <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="L2" t="str">
-        <x:v>Final Assessment</x:v>
+        <x:v>Final Assessment Retest after remediation</x:v>
       </x:c>
       <x:c r="M2" s="18" t="str">
-        <x:v>Explicit edge-case self-validation has not yet been demonstrated; final assessment is still required for S0-A completion.</x:v>
+        <x:v>Zero-boundary state handling and explicit edge-case self-validation.</x:v>
       </x:c>
       <x:c r="N2" s="18" t="str">
-        <x:v>Clean Part E retest PASS in 4:40. Correct input handling, branching, loop, helper function, scalar accumulation, and O(N)/O(1) analysis. Proceed to Part F.</x:v>
+        <x:v>Intermediate retest PASS in 4:40 established L3 evidence. Final Assessment Attempt 1 FAIL in 28:43 due important zero-case correctness errors. Keep L3/Provisional; remediate state-reset logic and edge-case validation, then use a new equivalent final-assessment problem.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" hidden="0" customHeight="1">
@@ -1439,7 +1525,7 @@
         <x:v>S0-A — C++ Basic Execution</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
-        <x:v>Part E intermediate assessment PASS; proceed to Part F final assessment</x:v>
+        <x:v>Part F final assessment attempt 1 FAIL; remediation + clean retest required</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
         <x:v>2026-09-11</x:v>
@@ -1492,10 +1578,10 @@
         <x:v>Current S0-A diagnostic</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>Intermediate PASS — L3 Provisional</x:v>
+        <x:v>Final FAIL — L3 Provisional</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
-        <x:v>Clean retest passed in 4:40; edge-case self-check not explicitly listed</x:v>
+        <x:v>Intermediate PASS retained; zero-boundary correctness failure in final assessment (28:43)</x:v>
       </x:c>
       <x:c r="D9" s="18" t="str">
         <x:v>2026-09-11</x:v>
@@ -1509,7 +1595,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>No Review Debt; final assessment pending</x:v>
+        <x:v>No Review Debt yet; immediate final-assessment retest pending after remediation</x:v>
       </x:c>
       <x:c r="D10" s="18" t="str">
         <x:v>2026-09-11</x:v>

</xml_diff>

<commit_message>
Update learning record after S0-A final retest FAIL
</commit_message>
<xml_diff>
--- a/records/CP_Learning_Record.xlsx
+++ b/records/CP_Learning_Record.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="R64d610c9006a4d3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="Rd4ac0ac7f8a94731"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="R2e4b3d4a5fd642d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="R6fe9475e86c04a26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="R2328eb3985e942e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="Rb69c87f518434876"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="Ra1d3b1592fbb4f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="Rc400ed334d5947b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="Rdd6433c599424e83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="Rd0179b8647ba48f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="R3a83d6784f264234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="Rd73a6ea8f3e94a0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="R3c91d9d715694ea4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="R4a93883ed54f4c59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="Rab531c4d4dba44f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="R2f3602a6d70b46f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="Rdc71d123b31c4228"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="Rb9e64f68e367494f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -781,6 +781,92 @@
         <x:v>Core O(N)/O(1) state-tracking idea is viable and sample/nonzero alternating cases work, but important zero cases fail. Counterexamples: N=1,[0] returns 1 instead of 0; [0,5,-3] returns 1 instead of 2. The duplicated unconditional `sum1 = 0;` inside the zero-product branch erases a valid new length-1 segment when previous value is zero and current value is nonzero. First-element logic also counts zero as a valid segment. First formal final-assessment FAIL; per v5.4 §39.1, convert this problem to learning mode, remediate, then reassess with a new equivalent problem.</x:v>
       </x:c>
     </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>S0-A — C++ Basic Execution</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Final Assessment — Retest 1</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Balance recovery count and maximum post-transaction balance</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>Reference execution + exhaustive small-case verification + randomized differential verification</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>R1</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>I2</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>Comparative / Provisional</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>CP_Calibration_Anchor_Registry_v1.1</x:v>
+      </x:c>
+      <x:c r="K5" t="str">
+        <x:v>Basic execution: input + conditional branching + loop + helper function + scalar state tracking + initial-state handling</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>Incomplete</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="N5"/>
+      <x:c r="O5" t="n">
+        <x:v>15.1</x:v>
+      </x:c>
+      <x:c r="P5"/>
+      <x:c r="Q5"/>
+      <x:c r="R5"/>
+      <x:c r="S5"/>
+      <x:c r="T5"/>
+      <x:c r="U5" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V5" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="W5" t="str">
+        <x:v>FAIL</x:v>
+      </x:c>
+      <x:c r="X5" t="str">
+        <x:v>Correctness</x:v>
+      </x:c>
+      <x:c r="Y5" t="str">
+        <x:v>Initial-state transition omitted: first transaction from balance 0 to positive is a recovery; no edge-case self-check; repeated boundary/initialization validation failure</x:v>
+      </x:c>
+      <x:c r="Z5" t="str">
+        <x:v>L3</x:v>
+      </x:c>
+      <x:c r="AA5" t="str">
+        <x:v>Provisional</x:v>
+      </x:c>
+      <x:c r="AB5" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="AC5" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="AD5" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="AE5" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AF5" t="str">
+        <x:v>Core O(N)/O(1) design and maximum-balance tracking are sound, but the special-case first iteration skips recovery detection. Counterexample: N=1, x=5 should output `1 5`, but submitted code outputs `0 5`. This is the second consecutive skill-related final-assessment FAIL on the same Learning Objective, with repeated boundary/edge-case validation weakness. Per v5.4 §39.2, pause formal retesting and perform diagnostic remediation before another new formal final-assessment problem.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -873,10 +959,10 @@
         <x:v>Incomplete</x:v>
       </x:c>
       <x:c r="H2" s="18" t="str">
-        <x:v>None</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="I2" s="18" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="J2" s="18" t="str">
         <x:v>Yes</x:v>
@@ -885,13 +971,13 @@
         <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="L2" t="str">
-        <x:v>Final Assessment Retest after remediation</x:v>
+        <x:v>Diagnostic remediation checkpoint before next Final Assessment</x:v>
       </x:c>
       <x:c r="M2" s="18" t="str">
-        <x:v>Zero-boundary state handling and explicit edge-case self-validation.</x:v>
+        <x:v>Repeated boundary/initial-state handling errors and absent explicit edge-case self-validation.</x:v>
       </x:c>
       <x:c r="N2" s="18" t="str">
-        <x:v>Intermediate retest PASS in 4:40 established L3 evidence. Final Assessment Attempt 1 FAIL in 28:43 due important zero-case correctness errors. Keep L3/Provisional; remediate state-reset logic and edge-case validation, then use a new equivalent final-assessment problem.</x:v>
+        <x:v>Intermediate retest PASS (4:40) still supports L3 implementation capability, but two consecutive skill-related final-assessment FAILs occurred (28:43, 15:06). Per v5.4 §39.2, stop simple retesting and perform diagnostic remediation. Medium Review Debt opened because the same boundary/edge-case validation error pattern repeated.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" hidden="0" customHeight="1">
@@ -1080,6 +1166,39 @@
       </x:c>
       <x:c r="K1" s="14" t="str">
         <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>S0-A — C++ Basic Execution</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>Repeated boundary/initial-state correctness errors and no explicit edge-case self-validation across two consecutive final assessments.</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>Diagnostic remediation: isolate initialization/first-step transitions, define state variables in words, and validate minimum/boundary cases before code lock; pass remediation checkpoint before new formal final-assessment retest.</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>Before next S0-A Final Assessment</x:v>
+      </x:c>
+      <x:c r="J2"/>
+      <x:c r="K2" t="str">
+        <x:v>Opened under v5.4 §28.3 because the same error type repeated. This is not a retroactive cancellation of the earlier intermediate PASS; S0-A remains incomplete.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1525,7 +1644,7 @@
         <x:v>S0-A — C++ Basic Execution</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
-        <x:v>Part F final assessment attempt 1 FAIL; remediation + clean retest required</x:v>
+        <x:v>Two consecutive Part F FAILs; diagnostic remediation required before another formal retest</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
         <x:v>2026-09-11</x:v>
@@ -1564,10 +1683,10 @@
         <x:v>Primary reasoning gap</x:v>
       </x:c>
       <x:c r="B8" s="18" t="str">
-        <x:v>correctness invariant / counterexample validation</x:v>
+        <x:v>boundary / initial-state correctness + counterexample validation</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
-        <x:v>Observed strongly in Baseline Problem C</x:v>
+        <x:v>Repeated in two consecutive S0-A final assessments</x:v>
       </x:c>
       <x:c r="D8" s="18" t="str">
         <x:v>2026-09-11</x:v>
@@ -1578,10 +1697,10 @@
         <x:v>Current S0-A diagnostic</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>Final FAIL — L3 Provisional</x:v>
+        <x:v>Final Retest 1 FAIL — L3 Provisional</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
-        <x:v>Intermediate PASS retained; zero-boundary correctness failure in final assessment (28:43)</x:v>
+        <x:v>First-transaction recovery omitted; T_solve 15:06; §39.2 remediation escalation active</x:v>
       </x:c>
       <x:c r="D9" s="18" t="str">
         <x:v>2026-09-11</x:v>
@@ -1592,10 +1711,10 @@
         <x:v>Review Debt</x:v>
       </x:c>
       <x:c r="B10" s="18" t="str">
-        <x:v>None</x:v>
+        <x:v>1 Open (Medium)</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>No Review Debt yet; immediate final-assessment retest pending after remediation</x:v>
+        <x:v>Repeated boundary/edge-case validation weakness in S0-A; prerequisite-blocking until remediation checkpoint</x:v>
       </x:c>
       <x:c r="D10" s="18" t="str">
         <x:v>2026-09-11</x:v>

</xml_diff>

<commit_message>
Record S0-A final retest 2 PASS in learning record
</commit_message>
<xml_diff>
--- a/records/CP_Learning_Record.xlsx
+++ b/records/CP_Learning_Record.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="Rd0179b8647ba48f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="R3a83d6784f264234"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="Rd73a6ea8f3e94a0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="R3c91d9d715694ea4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="R4a93883ed54f4c59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="Rab531c4d4dba44f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="R2f3602a6d70b46f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="Rdc71d123b31c4228"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="Rb9e64f68e367494f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="Rabd7a892e94a48fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="R4355f10e95614807"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="R981911e19bea488c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="R81504c1e4f904687"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="R377592fb091f4e59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="R1114d8f0c5824eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="Rf06ef37e01f347c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="Rc1fd5d97902942ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="R44d5be2fedf44670"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -867,6 +867,92 @@
         <x:v>Core O(N)/O(1) design and maximum-balance tracking are sound, but the special-case first iteration skips recovery detection. Counterexample: N=1, x=5 should output `1 5`, but submitted code outputs `0 5`. This is the second consecutive skill-related final-assessment FAIL on the same Learning Objective, with repeated boundary/edge-case validation weakness. Per v5.4 §39.2, pause formal retesting and perform diagnostic remediation before another new formal final-assessment problem.</x:v>
       </x:c>
     </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>S0-A — C++ Basic Execution</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Final Assessment — Retest 2</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>Record-break count and longest contiguous increasing segment</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>Exact-code compilation + sample/boundary execution + exhaustive small-case differential verification</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>R1</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>I2</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Comparative / Provisional</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>CP_Calibration_Anchor_Registry_v1.1</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>Basic execution: input + conditional branching + loop + helper function + scalar state tracking + initialization/boundary handling</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>Sufficient for Provisional</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>Immediate; Compiler/Debugger allowed</x:v>
+      </x:c>
+      <x:c r="N6"/>
+      <x:c r="O6" t="n">
+        <x:v>33.06666666666667</x:v>
+      </x:c>
+      <x:c r="P6"/>
+      <x:c r="Q6"/>
+      <x:c r="R6"/>
+      <x:c r="S6"/>
+      <x:c r="T6"/>
+      <x:c r="U6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V6" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="W6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="X6" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="Y6" t="str">
+        <x:v>No correctness error. Learner explicitly self-checked N=1 =&gt; 1 1. VS debugger use was permitted but actual use was not reported.</x:v>
+      </x:c>
+      <x:c r="Z6" t="str">
+        <x:v>L3</x:v>
+      </x:c>
+      <x:c r="AA6" t="str">
+        <x:v>Provisional</x:v>
+      </x:c>
+      <x:c r="AB6" t="str">
+        <x:v>Immediate; Compiler/Debugger allowed</x:v>
+      </x:c>
+      <x:c r="AC6" t="str">
+        <x:v>Resolved</x:v>
+      </x:c>
+      <x:c r="AD6" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="AE6" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AF6" t="str">
+        <x:v>Clean independent final retest after diagnostic remediation. Exact code compiled under C++17 and matched the sample, boundary executions, and exhaustive small-case differential checks. Record-break logic is correct because a new record is necessarily greater than the immediately previous value, so incrementing the current increasing-run length in that branch is valid. O(N) time and O(1) extra-space analyses are correct. Repeated initial/boundary-state weakness is considered remediated at immediate-evidence level; proceed to mandatory Part G Adaptive Extra Problem.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -956,28 +1042,28 @@
         <x:v>Immediate</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
-        <x:v>Incomplete</x:v>
+        <x:v>Sufficient for Provisional</x:v>
       </x:c>
       <x:c r="H2" s="18" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="I2" s="18" t="str">
-        <x:v>Medium</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="J2" s="18" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K2" s="18" t="str">
         <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="L2" t="str">
-        <x:v>Diagnostic remediation checkpoint before next Final Assessment</x:v>
+        <x:v>Part G Adaptive Extra Problem</x:v>
       </x:c>
       <x:c r="M2" s="18" t="str">
-        <x:v>Repeated boundary/initial-state handling errors and absent explicit edge-case self-validation.</x:v>
+        <x:v>No blocking correctness issue remains in immediate evidence; continue explicit edge-case validation habit.</x:v>
       </x:c>
       <x:c r="N2" s="18" t="str">
-        <x:v>Intermediate retest PASS (4:40) still supports L3 implementation capability, but two consecutive skill-related final-assessment FAILs occurred (28:43, 15:06). Per v5.4 §39.2, stop simple retesting and perform diagnostic remediation. Medium Review Debt opened because the same boundary/edge-case validation error pattern repeated.</x:v>
+        <x:v>Intermediate retest PASS and Final Retest 2 PASS. Diagnostic remediation checkpoint correctly articulated state meanings and first-transition handling. Medium Review Debt from repeated boundary/initial-state errors resolved after clean final retest. Long-term confidence remains Provisional pending delayed/mixed evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" hidden="0" customHeight="1">
@@ -1188,17 +1274,19 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="G2" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="H2" t="str">
-        <x:v>Diagnostic remediation: isolate initialization/first-step transitions, define state variables in words, and validate minimum/boundary cases before code lock; pass remediation checkpoint before new formal final-assessment retest.</x:v>
+        <x:v>Maintain mandatory explicit minimum/boundary-case self-check in future assessments; watch for recurrence in delayed/mixed evidence.</x:v>
       </x:c>
       <x:c r="I2" t="str">
-        <x:v>Before next S0-A Final Assessment</x:v>
-      </x:c>
-      <x:c r="J2"/>
+        <x:v>Delayed/Mixed Assessment</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
       <x:c r="K2" t="str">
-        <x:v>Opened under v5.4 §28.3 because the same error type repeated. This is not a retroactive cancellation of the earlier intermediate PASS; S0-A remains incomplete.</x:v>
+        <x:v>Diagnostic remediation checkpoint passed; subsequent Final Assessment Retest 2 passed independently with explicit N=1 edge-case check. Debt resolved, but recurrence should reopen debt.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1630,7 +1718,7 @@
         <x:v>Stage 0</x:v>
       </x:c>
       <x:c r="C4" s="18" t="str">
-        <x:v>S0-A in progress</x:v>
+        <x:v>S0-A Part F passed; Part G next</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
         <x:v>2026-09-11</x:v>
@@ -1644,7 +1732,7 @@
         <x:v>S0-A — C++ Basic Execution</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
-        <x:v>Two consecutive Part F FAILs; diagnostic remediation required before another formal retest</x:v>
+        <x:v>Part E PASS + Part F PASS; mandatory Adaptive Extra Problem pending</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
         <x:v>2026-09-11</x:v>
@@ -1686,7 +1774,7 @@
         <x:v>boundary / initial-state correctness + counterexample validation</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
-        <x:v>Repeated in two consecutive S0-A final assessments</x:v>
+        <x:v>Immediate remediation succeeded; monitor for recurrence in delayed/mixed evidence</x:v>
       </x:c>
       <x:c r="D8" s="18" t="str">
         <x:v>2026-09-11</x:v>
@@ -1697,10 +1785,10 @@
         <x:v>Current S0-A diagnostic</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>Final Retest 1 FAIL — L3 Provisional</x:v>
+        <x:v>Final Retest 2 PASS — L3 Provisional</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
-        <x:v>First-transaction recovery omitted; T_solve 15:06; §39.2 remediation escalation active</x:v>
+        <x:v>T_solve 33:04; explicit N=1 edge-case check; proceed to Part G</x:v>
       </x:c>
       <x:c r="D9" s="18" t="str">
         <x:v>2026-09-11</x:v>
@@ -1711,10 +1799,10 @@
         <x:v>Review Debt</x:v>
       </x:c>
       <x:c r="B10" s="18" t="str">
-        <x:v>1 Open (Medium)</x:v>
+        <x:v>0 Open</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>Repeated boundary/edge-case validation weakness in S0-A; prerequisite-blocking until remediation checkpoint</x:v>
+        <x:v>Prior Medium S0-A boundary/edge-case debt resolved after remediation + clean final retest</x:v>
       </x:c>
       <x:c r="D10" s="18" t="str">
         <x:v>2026-09-11</x:v>

</xml_diff>

<commit_message>
Record S0-B intermediate assessment PASS
</commit_message>
<xml_diff>
--- a/records/CP_Learning_Record.xlsx
+++ b/records/CP_Learning_Record.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="R8ad13d86ec39459a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="R7eeb04ecba7d4d5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="Rc7eb261593a148e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="Rccbb99da83d04601"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="Rc0e039fe131947f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="R3f032ec8ed70490a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="R41c476ae61a94407"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="R86ef23a71c7e4797"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="Rf2f0dd9dc43149fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="Rc1fde03d620a457c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="Red9d9ae3f57747b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="Rdf3950e533bd470f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="R883d7ccf99544bc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="R24e865e178134c4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="R455cdf781ea04a7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="R3db2977d84724d5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="R367ac3c819f74f45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="R7bf74ed596dc4e60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -924,6 +924,92 @@
         <x:v>Part G PASS; explicit N=1 checks; S0-A A-H complete.</x:v>
       </x:c>
     </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>S0-B — Basic Containers &amp; STL</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Intermediate Assessment — Attempt 1</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>Word Catalog — length then lexicographic sort; duplicates preserved</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Prevalidated reference + exhaustive/random differential; submitted C++17 compiled + sample/random differential</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>R1</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>I2</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>Comparative</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>vector/string + custom comparator + sort + duplicate preservation</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>Incomplete — Intermediate PASS; final not yet assessed</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="N8"/>
+      <x:c r="O8" t="n">
+        <x:v>10.2833</x:v>
+      </x:c>
+      <x:c r="P8"/>
+      <x:c r="Q8"/>
+      <x:c r="R8"/>
+      <x:c r="S8"/>
+      <x:c r="T8"/>
+      <x:c r="U8" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V8" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="W8" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="X8" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="Y8" t="str">
+        <x:v>None — minor explanation wording imprecision; signed/unsigned warning only</x:v>
+      </x:c>
+      <x:c r="Z8" t="str">
+        <x:v>L3</x:v>
+      </x:c>
+      <x:c r="AA8" t="str">
+        <x:v>Provisional</x:v>
+      </x:c>
+      <x:c r="AB8" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="AC8" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="AD8" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="AE8" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AF8" t="str">
+        <x:v>Correct code. Comparator uses length ascending then lexicographic ascending; duplicates retained. O(N log N) time and O(N) storage are valid with max string length 30. Explanation briefly said 'strings differ' where code checks 'lengths differ'; no correctness impact.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1032,16 +1118,16 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>L1</x:v>
+        <x:v>L3</x:v>
       </x:c>
       <x:c r="E3" t="str">
         <x:v>Provisional</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>Baseline</x:v>
+        <x:v>Immediate</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Intermediate PASS; Final not yet assessed</x:v>
       </x:c>
       <x:c r="H3" t="str">
         <x:v>None</x:v>
@@ -1050,19 +1136,19 @@
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="J3" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K3" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="L3" t="str">
-        <x:v>During S0-B</x:v>
+        <x:v>Final Assessment</x:v>
       </x:c>
       <x:c r="M3" t="str">
-        <x:v>vector/STL syntax and manipulation</x:v>
+        <x:v>Broader container/STL selection and transfer evidence still pending</x:v>
       </x:c>
       <x:c r="N3" t="str">
-        <x:v>Baseline A/B exposed gap.</x:v>
+        <x:v>Part E intermediate assessment PASS; canonical vector/string/sort/comparator implementation independently demonstrated.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1670,10 +1756,10 @@
         <x:v>Stage 0</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>S0-A complete; S0-B next</x:v>
+        <x:v>S0-B Part E intermediate PASS; final pending</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1684,10 +1770,10 @@
         <x:v>S0-B — Basic Containers &amp; STL</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>S0-A progression gate satisfied</x:v>
+        <x:v>Intermediate assessment PASS</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1723,13 +1809,13 @@
         <x:v>Primary next gap</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>vector/STL implementation</x:v>
+        <x:v>S0-B final/transfer evidence</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>Focus of S0-B</x:v>
+        <x:v>Broader container/STL selection still unverified</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
     </x:row>
     <x:row r="9">

</xml_diff>

<commit_message>
Record S0-B final assessment attempt 1 FAIL
</commit_message>
<xml_diff>
--- a/records/CP_Learning_Record.xlsx
+++ b/records/CP_Learning_Record.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="Rc1fde03d620a457c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="Red9d9ae3f57747b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="Rdf3950e533bd470f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="R883d7ccf99544bc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="R24e865e178134c4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="R455cdf781ea04a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="R3db2977d84724d5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="R367ac3c819f74f45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="R7bf74ed596dc4e60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="Rb18e490d2c984bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="R2156b0472a624a0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="Rba349085c8ef47ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="Redfb30ba205e4f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="Rc2eb5380fd2544ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="R956115e8de324a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="R8e9fdde10bdf4bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="Rd5bb143737c346cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="R12025444ee744ee2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1010,6 +1010,92 @@
         <x:v>Correct code. Comparator uses length ascending then lexicographic ascending; duplicates retained. O(N log N) time and O(N) storage are valid with max string length 30. Explanation briefly said 'strings differ' where code checks 'lengths differ'; no correctness impact.</x:v>
       </x:c>
     </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>S0-B — Basic Containers &amp; STL</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Final Assessment — Attempt 1</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>Priority List — priority desc, length asc, lexicographic asc; forward + exact reverse</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>Prevalidated reference + exhaustive/random differential; submitted C++17 compiled + sample output; explicit contract audit</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>R1</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>I2</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>Comparative / Provisional</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+      <x:c r="K9" t="str">
+        <x:v>vector&lt;pair&lt;string,int&gt;&gt; + custom comparator + sort/reverse + const-reference output-helper contract</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>Incomplete — Final FAIL; retest required</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="N9"/>
+      <x:c r="O9" t="n">
+        <x:v>24.3333</x:v>
+      </x:c>
+      <x:c r="P9"/>
+      <x:c r="Q9"/>
+      <x:c r="R9"/>
+      <x:c r="S9"/>
+      <x:c r="T9"/>
+      <x:c r="U9" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="W9" t="str">
+        <x:v>FAIL</x:v>
+      </x:c>
+      <x:c r="X9" t="str">
+        <x:v>Implementation</x:v>
+      </x:c>
+      <x:c r="Y9" t="str">
+        <x:v>Required print_records output function not implemented; comparator was named print_records instead. Container const-reference output interface therefore not demonstrated. Non-void comparator also emits fallthrough warning.</x:v>
+      </x:c>
+      <x:c r="Z9" t="str">
+        <x:v>L3</x:v>
+      </x:c>
+      <x:c r="AA9" t="str">
+        <x:v>Provisional</x:v>
+      </x:c>
+      <x:c r="AB9" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="AC9" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="AD9" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="AE9" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AF9" t="str">
+        <x:v>Sorting/output values are correct and complexity target is met, but an explicit assessed interface requirement was structurally missed. Same problem is now learning-only; use a new equivalent problem for retest.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1127,7 +1213,7 @@
         <x:v>Immediate</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>Intermediate PASS; Final not yet assessed</x:v>
+        <x:v>Intermediate PASS; Final Attempt 1 FAIL — retest required</x:v>
       </x:c>
       <x:c r="H3" t="str">
         <x:v>None</x:v>
@@ -1136,19 +1222,19 @@
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="J3" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="K3" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="L3" t="str">
-        <x:v>Final Assessment</x:v>
+        <x:v>Final Assessment Retest 1</x:v>
       </x:c>
       <x:c r="M3" t="str">
-        <x:v>Broader container/STL selection and transfer evidence still pending</x:v>
+        <x:v>Problem-contract/interface mapping: implement required output helper with container const-reference</x:v>
       </x:c>
       <x:c r="N3" t="str">
-        <x:v>Part E intermediate assessment PASS; canonical vector/string/sort/comparator implementation independently demonstrated.</x:v>
+        <x:v>Sorting/comparator/vector/pair/reverse logic is independently demonstrated; final attempt failed because the required print_records output function was not implemented.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1756,7 +1842,7 @@
         <x:v>Stage 0</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>S0-B Part E intermediate PASS; final pending</x:v>
+        <x:v>S0-B Part F final attempt 1 FAIL; retest pending</x:v>
       </x:c>
       <x:c r="D4" t="str">
         <x:v>2026-09-15</x:v>
@@ -1770,7 +1856,7 @@
         <x:v>S0-B — Basic Containers &amp; STL</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Intermediate assessment PASS</x:v>
+        <x:v>Intermediate PASS; Final retest required</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>2026-09-15</x:v>
@@ -1809,10 +1895,10 @@
         <x:v>Primary next gap</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>S0-B final/transfer evidence</x:v>
+        <x:v>S0-B interface-contract retest</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>Broader container/STL selection still unverified</x:v>
+        <x:v>Sorting logic correct; required const-ref print helper was missed</x:v>
       </x:c>
       <x:c r="D8" t="str">
         <x:v>2026-09-15</x:v>

</xml_diff>

<commit_message>
Record v5.5 External CP Extra conditional pass
</commit_message>
<xml_diff>
--- a/records/CP_Learning_Record.xlsx
+++ b/records/CP_Learning_Record.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="Rb0316a5798d54f36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="Ra12cd6f65db644ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="Raf874f697b214626"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="R8690db1676924cd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="R4097597294174885"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="R9397512ebef84164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="Raa43339e005e4f11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="R66f93c63fef84d5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="Ra2990a0f9bc44e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="1" r:id="Re4bd5171355a4942"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="2" r:id="Rba6a2571d8284b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mastery" sheetId="3" r:id="Rcf7b571c6a7b4245"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision_Coverage" sheetId="4" r:id="R19628492a4474f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Debt" sheetId="5" r:id="Rbedd507439af4da6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="6" r:id="R2aef51e4f0b24a0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks" sheetId="7" r:id="R366dbf8ca5ac41ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness" sheetId="8" r:id="R66bd2c5665034c98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="R3096cc727bc04567"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1354,6 +1354,92 @@
         <x:v>Code is correct and satisfies the required normalize(vector&lt;string&gt;&amp;) in-place contract. Correct total complexity uses L=sum of word lengths: O(L) time and O(L) total storage including input, O(1) auxiliary space. One non-blocking signed/unsigned loop warning. Fresh equivalent reassessment required for the complexity-analysis objective.</x:v>
       </x:c>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>S0-B — Basic Containers &amp; STL</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>v5.5 Extra Problem — External CP</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>AtCoder ABC104 B — AcCepted</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>Official AtCoder judge/problem statement; submitted C++17 compiled locally; targeted counterexample audit</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>R1</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>I1</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>Comparative / Provisional</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+      <x:c r="K13" t="str">
+        <x:v>string indexing + conditional validation + uppercase/lowercase checks + bounded scan</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>Complete — Progression Gate previously satisfied; post-completion External Extra evidence</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="N13"/>
+      <x:c r="O13" t="n">
+        <x:v>24.95</x:v>
+      </x:c>
+      <x:c r="P13"/>
+      <x:c r="Q13"/>
+      <x:c r="R13"/>
+      <x:c r="S13"/>
+      <x:c r="T13"/>
+      <x:c r="U13" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V13" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="W13" t="str">
+        <x:v>CONDITIONAL PASS</x:v>
+      </x:c>
+      <x:c r="X13" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="Y13" t="str">
+        <x:v>Local implementation bug: uppercase 'Z' is never checked because loop condition c != 'Z' stops before Z</x:v>
+      </x:c>
+      <x:c r="Z13" t="str">
+        <x:v>L3</x:v>
+      </x:c>
+      <x:c r="AA13" t="str">
+        <x:v>Provisional</x:v>
+      </x:c>
+      <x:c r="AB13" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="AC13" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="AD13" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="AE13" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AF13" t="str">
+        <x:v>Core solution structure and O(|S|) time / O(|S|) total storage analysis are correct. One-line boundary fix is sufficient: the uppercase scan must include 'Z' (e.g. c &lt;= 'Z') or use an equivalent uppercase test. Counterexample: AcCZ should be WA but submitted code prints AC. User edge cases AccC-&gt;WA and AcCc-&gt;AC are correct. Fresh equivalent full-PASS evidence is required; this does not revoke the prior S0-B progression gate.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1486,13 +1572,13 @@
         <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="L3" t="str">
-        <x:v>Fresh equivalent Extra / S0-C transfer check</x:v>
+        <x:v>Fresh equivalent Extra / S0-C transfer check + mixed S0-B review</x:v>
       </x:c>
       <x:c r="M3" t="str">
-        <x:v>Complexity accounting for non-constant library operations and distinguishing N from total input size L</x:v>
+        <x:v>Primary: complexity accounting for non-constant library operations and N vs total input length L; secondary: exact boundary handling in character classification</x:v>
       </x:c>
       <x:c r="N3" t="str">
-        <x:v>A-H progression gate remains satisfied. Post-completion v5.5 GPT-generated Extra: code correct, but assessment FAIL on complexity explanation; Medium Review Debt opened. Confidence remains Provisional.</x:v>
+        <x:v>A-H progression gate remains satisfied. Post-completion v5.5 GPT-generated Extra FAIL opened Medium complexity debt. External CP Extra (AtCoder ABC104 B) received CONDITIONAL PASS: solution structure and complexity were correct, but uppercase 'Z' was omitted by a one-line loop-bound bug. An additional Low implementation debt is open. Overall debt severity remains Medium; Confidence remains Provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1747,6 +1833,39 @@
         <x:v>Post-completion Extra FAIL does not revoke the prior S0-B progression gate; debt tracks the unresolved complexity-analysis objective.</x:v>
       </x:c>
     </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>S0-B — Basic Containers &amp; STL</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>Local uppercase-boundary implementation bug in External Extra: 'Z' omitted from uppercase scan</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Reassess exact character-boundary validation on a fresh equivalent problem; require full PASS without hints</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>Fresh equivalent Extra / mixed S0-B review</x:v>
+      </x:c>
+      <x:c r="J4"/>
+      <x:c r="K4" t="str">
+        <x:v>CONDITIONAL PASS creates Review Debt until a clean full PASS. Existing Medium complexity debt remains separately open.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>